<commit_message>
updated comparisons for per QID fisher test
</commit_message>
<xml_diff>
--- a/eval/learning-curve/results/statistical_tests_new30.xlsx
+++ b/eval/learning-curve/results/statistical_tests_new30.xlsx
@@ -5413,7 +5413,7 @@
         <v>0.0523</v>
       </c>
       <c r="I3" t="n">
-        <v>0.369</v>
+        <v>0.131</v>
       </c>
     </row>
     <row r="4">
@@ -5783,7 +5783,7 @@
         <v>0.104</v>
       </c>
       <c r="I13" t="n">
-        <v>0.417</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -5857,7 +5857,7 @@
         <v>0.0575</v>
       </c>
       <c r="I15" t="n">
-        <v>0.369</v>
+        <v>0.863</v>
       </c>
     </row>
     <row r="16">
@@ -5931,7 +5931,7 @@
         <v>0.0692</v>
       </c>
       <c r="I17" t="n">
-        <v>0.369</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="18">
@@ -5968,7 +5968,7 @@
         <v>0.219</v>
       </c>
       <c r="I18" t="n">
-        <v>0.979</v>
+        <v>0.831</v>
       </c>
     </row>
     <row r="19">
@@ -6005,7 +6005,7 @@
         <v>0.245</v>
       </c>
       <c r="I19" t="n">
-        <v>0.979</v>
+        <v>0.612</v>
       </c>
     </row>
     <row r="20">
@@ -6301,7 +6301,7 @@
         <v>0.664</v>
       </c>
       <c r="I27" t="n">
-        <v>1</v>
+        <v>0.9419999999999999</v>
       </c>
     </row>
     <row r="28">
@@ -6338,7 +6338,7 @@
         <v>0.216</v>
       </c>
       <c r="I28" t="n">
-        <v>0.979</v>
+        <v>0.802</v>
       </c>
     </row>
     <row r="29">
@@ -6523,7 +6523,7 @@
         <v>0.141</v>
       </c>
       <c r="I33" t="n">
-        <v>0.979</v>
+        <v>0.608</v>
       </c>
     </row>
     <row r="34">
@@ -6560,7 +6560,7 @@
         <v>0.0496</v>
       </c>
       <c r="I34" t="n">
-        <v>0.265</v>
+        <v>0.372</v>
       </c>
     </row>
     <row r="35">
@@ -6819,7 +6819,7 @@
         <v>0.5669999999999999</v>
       </c>
       <c r="I41" t="n">
-        <v>1</v>
+        <v>0.945</v>
       </c>
     </row>
     <row r="42">
@@ -6967,7 +6967,7 @@
         <v>0.0293</v>
       </c>
       <c r="I45" t="n">
-        <v>0.234</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="46">
@@ -7041,7 +7041,7 @@
         <v>0.008359999999999999</v>
       </c>
       <c r="I47" t="n">
-        <v>0.134</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="48">
@@ -7115,7 +7115,7 @@
         <v>0.0707</v>
       </c>
       <c r="I49" t="n">
-        <v>0.283</v>
+        <v>0.353</v>
       </c>
     </row>
     <row r="50">
@@ -7152,7 +7152,7 @@
         <v>0.763</v>
       </c>
       <c r="I50" t="n">
-        <v>1</v>
+        <v>0.984</v>
       </c>
     </row>
     <row r="51">
@@ -7189,7 +7189,7 @@
         <v>0.158</v>
       </c>
       <c r="I51" t="n">
-        <v>0.631</v>
+        <v>0.339</v>
       </c>
     </row>
     <row r="52">
@@ -7226,7 +7226,7 @@
         <v>0.485</v>
       </c>
       <c r="I52" t="n">
-        <v>0.776</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -7263,7 +7263,7 @@
         <v>0.481</v>
       </c>
       <c r="I53" t="n">
-        <v>0.776</v>
+        <v>0.722</v>
       </c>
     </row>
     <row r="54">
@@ -7300,7 +7300,7 @@
         <v>0.427</v>
       </c>
       <c r="I54" t="n">
-        <v>0.776</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -7411,7 +7411,7 @@
         <v>0.321</v>
       </c>
       <c r="I57" t="n">
-        <v>0.776</v>
+        <v>0.535</v>
       </c>
     </row>
     <row r="58">
@@ -7448,7 +7448,7 @@
         <v>0.463</v>
       </c>
       <c r="I58" t="n">
-        <v>0.776</v>
+        <v>0.928</v>
       </c>
     </row>
     <row r="59">
@@ -7559,7 +7559,7 @@
         <v>0.0242</v>
       </c>
       <c r="I61" t="n">
-        <v>0.129</v>
+        <v>0.363</v>
       </c>
     </row>
     <row r="62">
@@ -7633,7 +7633,7 @@
         <v>0.0124</v>
       </c>
       <c r="I63" t="n">
-        <v>0.09950000000000001</v>
+        <v>0.186</v>
       </c>
     </row>
     <row r="64">
@@ -7670,7 +7670,7 @@
         <v>0.431</v>
       </c>
       <c r="I64" t="n">
-        <v>0.776</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
@@ -7707,7 +7707,7 @@
         <v>0.006</v>
       </c>
       <c r="I65" t="n">
-        <v>0.0961</v>
+        <v>0.0419</v>
       </c>
     </row>
     <row r="66">
@@ -7781,7 +7781,7 @@
         <v>0.0105</v>
       </c>
       <c r="I67" t="n">
-        <v>0.0843</v>
+        <v>0.0788</v>
       </c>
     </row>
     <row r="68">
@@ -7855,7 +7855,7 @@
         <v>1.88e-11</v>
       </c>
       <c r="I69" t="n">
-        <v>3e-10</v>
+        <v>9.4e-11</v>
       </c>
     </row>
     <row r="70">
@@ -8077,7 +8077,7 @@
         <v>0.0539</v>
       </c>
       <c r="I75" t="n">
-        <v>0.287</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="76">
@@ -8299,7 +8299,7 @@
         <v>0.12</v>
       </c>
       <c r="I81" t="n">
-        <v>0.482</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="82">
@@ -8336,7 +8336,7 @@
         <v>0.487</v>
       </c>
       <c r="I82" t="n">
-        <v>1</v>
+        <v>0.913</v>
       </c>
     </row>
     <row r="83">
@@ -8373,7 +8373,7 @@
         <v>0.0699</v>
       </c>
       <c r="I83" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.524</v>
       </c>
     </row>
     <row r="84">
@@ -8447,7 +8447,7 @@
         <v>5.65e-06</v>
       </c>
       <c r="I85" t="n">
-        <v>9.03e-05</v>
+        <v>2.82e-05</v>
       </c>
     </row>
     <row r="86">
@@ -8669,7 +8669,7 @@
         <v>0.167</v>
       </c>
       <c r="I91" t="n">
-        <v>0.669</v>
+        <v>0.754</v>
       </c>
     </row>
     <row r="92">
@@ -8706,7 +8706,7 @@
         <v>0.42</v>
       </c>
       <c r="I92" t="n">
-        <v>1</v>
+        <v>0.802</v>
       </c>
     </row>
     <row r="93">
@@ -8891,7 +8891,7 @@
         <v>0.162</v>
       </c>
       <c r="I97" t="n">
-        <v>0.669</v>
+        <v>0.608</v>
       </c>
     </row>
     <row r="98">
@@ -8928,7 +8928,7 @@
         <v>0.489</v>
       </c>
       <c r="I98" t="n">
-        <v>1</v>
+        <v>0.8149999999999999</v>
       </c>
     </row>
     <row r="99">
@@ -9039,7 +9039,7 @@
         <v>0.00466</v>
       </c>
       <c r="I101" t="n">
-        <v>0.0746</v>
+        <v>0.0175</v>
       </c>
     </row>
     <row r="102">
@@ -9187,7 +9187,7 @@
         <v>0.242</v>
       </c>
       <c r="I105" t="n">
-        <v>0.97</v>
+        <v>0.907</v>
       </c>
     </row>
     <row r="106">
@@ -9261,7 +9261,7 @@
         <v>0.208</v>
       </c>
       <c r="I107" t="n">
-        <v>0.97</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108">
@@ -9409,7 +9409,7 @@
         <v>0.605</v>
       </c>
       <c r="I111" t="n">
-        <v>1</v>
+        <v>0.826</v>
       </c>
     </row>
     <row r="112">
@@ -9483,7 +9483,7 @@
         <v>0.141</v>
       </c>
       <c r="I113" t="n">
-        <v>0.97</v>
+        <v>0.486</v>
       </c>
     </row>
     <row r="114">
@@ -9557,7 +9557,7 @@
         <v>0.0436</v>
       </c>
       <c r="I115" t="n">
-        <v>0.174</v>
+        <v>0.327</v>
       </c>
     </row>
     <row r="116">
@@ -9631,7 +9631,7 @@
         <v>3.32e-09</v>
       </c>
       <c r="I117" t="n">
-        <v>5.32e-08</v>
+        <v>1.66e-08</v>
       </c>
     </row>
     <row r="118">
@@ -9742,7 +9742,7 @@
         <v>0.348</v>
       </c>
       <c r="I120" t="n">
-        <v>0.929</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="121">
@@ -9779,7 +9779,7 @@
         <v>0.0584</v>
       </c>
       <c r="I121" t="n">
-        <v>0.187</v>
+        <v>0.219</v>
       </c>
     </row>
     <row r="122">
@@ -9853,7 +9853,7 @@
         <v>0.0398</v>
       </c>
       <c r="I123" t="n">
-        <v>0.174</v>
+        <v>0.5620000000000001</v>
       </c>
     </row>
     <row r="124">
@@ -9927,7 +9927,7 @@
         <v>0.711</v>
       </c>
       <c r="I125" t="n">
-        <v>1</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="126">
@@ -10075,7 +10075,7 @@
         <v>0.0229</v>
       </c>
       <c r="I129" t="n">
-        <v>0.174</v>
+        <v>0.0859</v>
       </c>
     </row>
     <row r="130">
@@ -10149,7 +10149,7 @@
         <v>0.0105</v>
       </c>
       <c r="I131" t="n">
-        <v>0.169</v>
+        <v>0.0788</v>
       </c>
     </row>
     <row r="132">
@@ -10445,7 +10445,7 @@
         <v>0.43</v>
       </c>
       <c r="I139" t="n">
-        <v>1</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="140">
@@ -10667,7 +10667,7 @@
         <v>0.196</v>
       </c>
       <c r="I145" t="n">
-        <v>1</v>
+        <v>0.547</v>
       </c>
     </row>
     <row r="146">
@@ -10704,7 +10704,7 @@
         <v>0.123</v>
       </c>
       <c r="I146" t="n">
-        <v>0.984</v>
+        <v>0.831</v>
       </c>
     </row>
     <row r="147">
@@ -10741,7 +10741,7 @@
         <v>0.0699</v>
       </c>
       <c r="I147" t="n">
-        <v>0.984</v>
+        <v>0.524</v>
       </c>
     </row>
     <row r="148">
@@ -11037,7 +11037,7 @@
         <v>0.656</v>
       </c>
       <c r="I155" t="n">
-        <v>1</v>
+        <v>0.9419999999999999</v>
       </c>
     </row>
     <row r="156">
@@ -11074,7 +11074,7 @@
         <v>0.428</v>
       </c>
       <c r="I156" t="n">
-        <v>1</v>
+        <v>0.802</v>
       </c>
     </row>
     <row r="157">
@@ -11259,7 +11259,7 @@
         <v>0.266</v>
       </c>
       <c r="I161" t="n">
-        <v>1</v>
+        <v>0.656</v>
       </c>
     </row>
     <row r="162">
@@ -11296,7 +11296,7 @@
         <v>0.489</v>
       </c>
       <c r="I162" t="n">
-        <v>1</v>
+        <v>0.8149999999999999</v>
       </c>
     </row>
     <row r="163">
@@ -11555,7 +11555,7 @@
         <v>0.5669999999999999</v>
       </c>
       <c r="I169" t="n">
-        <v>1</v>
+        <v>0.945</v>
       </c>
     </row>
     <row r="170">
@@ -11703,7 +11703,7 @@
         <v>0.232</v>
       </c>
       <c r="I173" t="n">
-        <v>1</v>
+        <v>0.868</v>
       </c>
     </row>
     <row r="174">
@@ -11777,7 +11777,7 @@
         <v>0.182</v>
       </c>
       <c r="I175" t="n">
-        <v>1</v>
+        <v>0.826</v>
       </c>
     </row>
     <row r="176">
@@ -11851,7 +11851,7 @@
         <v>0.438</v>
       </c>
       <c r="I177" t="n">
-        <v>1</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="178">
@@ -11888,7 +11888,7 @@
         <v>0.498</v>
       </c>
       <c r="I178" t="n">
-        <v>0.885</v>
+        <v>0.984</v>
       </c>
     </row>
     <row r="179">
@@ -11925,7 +11925,7 @@
         <v>0.0436</v>
       </c>
       <c r="I179" t="n">
-        <v>0.698</v>
+        <v>0.327</v>
       </c>
     </row>
     <row r="180">
@@ -11999,7 +11999,7 @@
         <v>0.481</v>
       </c>
       <c r="I181" t="n">
-        <v>0.885</v>
+        <v>0.722</v>
       </c>
     </row>
     <row r="182">
@@ -12073,7 +12073,7 @@
         <v>0.484</v>
       </c>
       <c r="I183" t="n">
-        <v>0.885</v>
+        <v>1</v>
       </c>
     </row>
     <row r="184">
@@ -12110,7 +12110,7 @@
         <v>0.737</v>
       </c>
       <c r="I184" t="n">
-        <v>1</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="185">
@@ -12147,7 +12147,7 @@
         <v>0.321</v>
       </c>
       <c r="I185" t="n">
-        <v>0.885</v>
+        <v>0.535</v>
       </c>
     </row>
     <row r="186">
@@ -12184,7 +12184,7 @@
         <v>0.804</v>
       </c>
       <c r="I186" t="n">
-        <v>1</v>
+        <v>0.928</v>
       </c>
     </row>
     <row r="187">
@@ -12221,7 +12221,7 @@
         <v>0.465</v>
       </c>
       <c r="I187" t="n">
-        <v>0.885</v>
+        <v>0.868</v>
       </c>
     </row>
     <row r="188">
@@ -12295,7 +12295,7 @@
         <v>0.285</v>
       </c>
       <c r="I189" t="n">
-        <v>0.885</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="190">
@@ -12369,7 +12369,7 @@
         <v>0.459</v>
       </c>
       <c r="I191" t="n">
-        <v>0.885</v>
+        <v>1</v>
       </c>
     </row>
     <row r="192">
@@ -12406,7 +12406,7 @@
         <v>0.5610000000000001</v>
       </c>
       <c r="I192" t="n">
-        <v>0.898</v>
+        <v>1</v>
       </c>
     </row>
     <row r="193">
@@ -12443,7 +12443,7 @@
         <v>0.135</v>
       </c>
       <c r="I193" t="n">
-        <v>0.885</v>
+        <v>0.225</v>
       </c>
     </row>
     <row r="194">
@@ -12517,7 +12517,7 @@
         <v>0.299</v>
       </c>
       <c r="I195" t="n">
-        <v>1</v>
+        <v>0.448</v>
       </c>
     </row>
     <row r="196">
@@ -12591,7 +12591,7 @@
         <v>2.36e-12</v>
       </c>
       <c r="I197" t="n">
-        <v>3.77e-11</v>
+        <v>1.77e-11</v>
       </c>
     </row>
     <row r="198">
@@ -12813,7 +12813,7 @@
         <v>0.18</v>
       </c>
       <c r="I203" t="n">
-        <v>1</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="204">
@@ -13035,7 +13035,7 @@
         <v>0.604</v>
       </c>
       <c r="I209" t="n">
-        <v>1</v>
+        <v>0.647</v>
       </c>
     </row>
     <row r="210">
@@ -13109,7 +13109,7 @@
         <v>0.58</v>
       </c>
       <c r="I211" t="n">
-        <v>1</v>
+        <v>0.828</v>
       </c>
     </row>
     <row r="212">
@@ -13183,7 +13183,7 @@
         <v>4.34e-06</v>
       </c>
       <c r="I213" t="n">
-        <v>6.95e-05</v>
+        <v>2.82e-05</v>
       </c>
     </row>
     <row r="214">
@@ -13405,7 +13405,7 @@
         <v>0.335</v>
       </c>
       <c r="I219" t="n">
-        <v>1</v>
+        <v>0.754</v>
       </c>
     </row>
     <row r="220">
@@ -13442,7 +13442,7 @@
         <v>0.42</v>
       </c>
       <c r="I220" t="n">
-        <v>1</v>
+        <v>0.802</v>
       </c>
     </row>
     <row r="221">
@@ -13627,7 +13627,7 @@
         <v>0.592</v>
       </c>
       <c r="I225" t="n">
-        <v>1</v>
+        <v>0.823</v>
       </c>
     </row>
     <row r="226">
@@ -13664,7 +13664,7 @@
         <v>0.489</v>
       </c>
       <c r="I226" t="n">
-        <v>1</v>
+        <v>0.8149999999999999</v>
       </c>
     </row>
     <row r="227">
@@ -13775,7 +13775,7 @@
         <v>0.00466</v>
       </c>
       <c r="I229" t="n">
-        <v>0.0746</v>
+        <v>0.0175</v>
       </c>
     </row>
     <row r="230">
@@ -13923,7 +13923,7 @@
         <v>0.242</v>
       </c>
       <c r="I233" t="n">
-        <v>1</v>
+        <v>0.907</v>
       </c>
     </row>
     <row r="234">
@@ -14071,7 +14071,7 @@
         <v>0.232</v>
       </c>
       <c r="I237" t="n">
-        <v>1</v>
+        <v>0.868</v>
       </c>
     </row>
     <row r="238">
@@ -14145,7 +14145,7 @@
         <v>0.605</v>
       </c>
       <c r="I239" t="n">
-        <v>1</v>
+        <v>0.826</v>
       </c>
     </row>
     <row r="240">
@@ -14256,7 +14256,7 @@
         <v>0.772</v>
       </c>
       <c r="I242" t="n">
-        <v>1</v>
+        <v>0.984</v>
       </c>
     </row>
     <row r="243">
@@ -14367,7 +14367,7 @@
         <v>2.33e-09</v>
       </c>
       <c r="I245" t="n">
-        <v>3.72e-08</v>
+        <v>1.66e-08</v>
       </c>
     </row>
     <row r="246">
@@ -14478,7 +14478,7 @@
         <v>0.737</v>
       </c>
       <c r="I248" t="n">
-        <v>1</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="249">
@@ -14515,7 +14515,7 @@
         <v>0.0584</v>
       </c>
       <c r="I249" t="n">
-        <v>0.467</v>
+        <v>0.219</v>
       </c>
     </row>
     <row r="250">
@@ -14552,7 +14552,7 @@
         <v>0.804</v>
       </c>
       <c r="I250" t="n">
-        <v>1</v>
+        <v>0.928</v>
       </c>
     </row>
     <row r="251">
@@ -14589,7 +14589,7 @@
         <v>0.21</v>
       </c>
       <c r="I251" t="n">
-        <v>0.841</v>
+        <v>0.5620000000000001</v>
       </c>
     </row>
     <row r="252">
@@ -14663,7 +14663,7 @@
         <v>0.173</v>
       </c>
       <c r="I253" t="n">
-        <v>0.841</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="254">
@@ -14811,7 +14811,7 @@
         <v>0.534</v>
       </c>
       <c r="I257" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
     </row>
     <row r="258">
@@ -14885,7 +14885,7 @@
         <v>0.145</v>
       </c>
       <c r="I259" t="n">
-        <v>1</v>
+        <v>0.272</v>
       </c>
     </row>
     <row r="260">
@@ -15181,7 +15181,7 @@
         <v>0.18</v>
       </c>
       <c r="I267" t="n">
-        <v>1</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="268">
@@ -15403,7 +15403,7 @@
         <v>0.438</v>
       </c>
       <c r="I273" t="n">
-        <v>1</v>
+        <v>0.547</v>
       </c>
     </row>
     <row r="274">
@@ -15477,7 +15477,7 @@
         <v>0.51</v>
       </c>
       <c r="I275" t="n">
-        <v>1</v>
+        <v>0.828</v>
       </c>
     </row>
     <row r="276">
@@ -15773,7 +15773,7 @@
         <v>0.335</v>
       </c>
       <c r="I283" t="n">
-        <v>1</v>
+        <v>0.754</v>
       </c>
     </row>
     <row r="284">
@@ -15995,7 +15995,7 @@
         <v>0.665</v>
       </c>
       <c r="I289" t="n">
-        <v>1</v>
+        <v>0.823</v>
       </c>
     </row>
     <row r="290">
@@ -16032,7 +16032,7 @@
         <v>0.109</v>
       </c>
       <c r="I290" t="n">
-        <v>0.754</v>
+        <v>0.545</v>
       </c>
     </row>
     <row r="291">
@@ -16106,7 +16106,7 @@
         <v>0.462</v>
       </c>
       <c r="I292" t="n">
-        <v>0.805</v>
+        <v>1</v>
       </c>
     </row>
     <row r="293">
@@ -16180,7 +16180,7 @@
         <v>0.556</v>
       </c>
       <c r="I294" t="n">
-        <v>0.805</v>
+        <v>1</v>
       </c>
     </row>
     <row r="295">
@@ -16217,7 +16217,7 @@
         <v>0.343</v>
       </c>
       <c r="I295" t="n">
-        <v>0.754</v>
+        <v>1</v>
       </c>
     </row>
     <row r="296">
@@ -16254,7 +16254,7 @@
         <v>0.604</v>
       </c>
       <c r="I296" t="n">
-        <v>0.805</v>
+        <v>1</v>
       </c>
     </row>
     <row r="297">
@@ -16291,7 +16291,7 @@
         <v>0.242</v>
       </c>
       <c r="I297" t="n">
-        <v>0.754</v>
+        <v>0.907</v>
       </c>
     </row>
     <row r="298">
@@ -16328,7 +16328,7 @@
         <v>0.785</v>
       </c>
       <c r="I298" t="n">
-        <v>0.966</v>
+        <v>1</v>
       </c>
     </row>
     <row r="299">
@@ -16365,7 +16365,7 @@
         <v>0.542</v>
       </c>
       <c r="I299" t="n">
-        <v>0.805</v>
+        <v>1</v>
       </c>
     </row>
     <row r="300">
@@ -16402,7 +16402,7 @@
         <v>0.377</v>
       </c>
       <c r="I300" t="n">
-        <v>0.754</v>
+        <v>1</v>
       </c>
     </row>
     <row r="301">
@@ -16439,7 +16439,7 @@
         <v>0.232</v>
       </c>
       <c r="I301" t="n">
-        <v>0.754</v>
+        <v>0.868</v>
       </c>
     </row>
     <row r="302">
@@ -16513,7 +16513,7 @@
         <v>0.342</v>
       </c>
       <c r="I303" t="n">
-        <v>0.754</v>
+        <v>0.826</v>
       </c>
     </row>
     <row r="304">
@@ -16550,7 +16550,7 @@
         <v>0.273</v>
       </c>
       <c r="I304" t="n">
-        <v>0.754</v>
+        <v>1</v>
       </c>
     </row>
     <row r="305">
@@ -16587,7 +16587,7 @@
         <v>0.0134</v>
       </c>
       <c r="I305" t="n">
-        <v>0.214</v>
+        <v>0.101</v>
       </c>
     </row>
     <row r="306">
@@ -16624,7 +16624,7 @@
         <v>0.5659999999999999</v>
       </c>
       <c r="I306" t="n">
-        <v>0.728</v>
+        <v>0.984</v>
       </c>
     </row>
     <row r="307">
@@ -16661,7 +16661,7 @@
         <v>0.628</v>
       </c>
       <c r="I307" t="n">
-        <v>0.728</v>
+        <v>0.856</v>
       </c>
     </row>
     <row r="308">
@@ -16698,7 +16698,7 @@
         <v>0.203</v>
       </c>
       <c r="I308" t="n">
-        <v>0.728</v>
+        <v>1</v>
       </c>
     </row>
     <row r="309">
@@ -16735,7 +16735,7 @@
         <v>0.593</v>
       </c>
       <c r="I309" t="n">
-        <v>0.728</v>
+        <v>0.8090000000000001</v>
       </c>
     </row>
     <row r="310">
@@ -16772,7 +16772,7 @@
         <v>0.475</v>
       </c>
       <c r="I310" t="n">
-        <v>0.728</v>
+        <v>1</v>
       </c>
     </row>
     <row r="311">
@@ -16809,7 +16809,7 @@
         <v>0.468</v>
       </c>
       <c r="I311" t="n">
-        <v>0.728</v>
+        <v>1</v>
       </c>
     </row>
     <row r="312">
@@ -16846,7 +16846,7 @@
         <v>0.731</v>
       </c>
       <c r="I312" t="n">
-        <v>0.779</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="313">
@@ -16883,7 +16883,7 @@
         <v>0.0584</v>
       </c>
       <c r="I313" t="n">
-        <v>0.467</v>
+        <v>0.219</v>
       </c>
     </row>
     <row r="314">
@@ -16920,7 +16920,7 @@
         <v>0.622</v>
       </c>
       <c r="I314" t="n">
-        <v>0.728</v>
+        <v>0.928</v>
       </c>
     </row>
     <row r="315">
@@ -16957,7 +16957,7 @@
         <v>0.21</v>
       </c>
       <c r="I315" t="n">
-        <v>0.728</v>
+        <v>0.5620000000000001</v>
       </c>
     </row>
     <row r="316">
@@ -16994,7 +16994,7 @@
         <v>0.637</v>
       </c>
       <c r="I316" t="n">
-        <v>0.728</v>
+        <v>1</v>
       </c>
     </row>
     <row r="317">
@@ -17031,7 +17031,7 @@
         <v>0.285</v>
       </c>
       <c r="I317" t="n">
-        <v>0.728</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="318">
@@ -17105,7 +17105,7 @@
         <v>0.466</v>
       </c>
       <c r="I319" t="n">
-        <v>0.728</v>
+        <v>1</v>
       </c>
     </row>
     <row r="320">
@@ -17142,7 +17142,7 @@
         <v>0.584</v>
       </c>
       <c r="I320" t="n">
-        <v>0.728</v>
+        <v>1</v>
       </c>
     </row>
     <row r="321">
@@ -17179,7 +17179,7 @@
         <v>0.00839</v>
       </c>
       <c r="I321" t="n">
-        <v>0.134</v>
+        <v>0.0419</v>
       </c>
     </row>
     <row r="322">
@@ -17253,7 +17253,7 @@
         <v>0.0523</v>
       </c>
       <c r="I323" t="n">
-        <v>0.419</v>
+        <v>0.131</v>
       </c>
     </row>
     <row r="324">
@@ -17327,7 +17327,7 @@
         <v>3.42e-09</v>
       </c>
       <c r="I325" t="n">
-        <v>5.47e-08</v>
+        <v>1.28e-08</v>
       </c>
     </row>
     <row r="326">
@@ -17364,7 +17364,7 @@
         <v>0.399</v>
       </c>
       <c r="I326" t="n">
-        <v>0.969</v>
+        <v>1</v>
       </c>
     </row>
     <row r="327">
@@ -17475,7 +17475,7 @@
         <v>0.424</v>
       </c>
       <c r="I329" t="n">
-        <v>0.969</v>
+        <v>1</v>
       </c>
     </row>
     <row r="330">
@@ -17549,7 +17549,7 @@
         <v>0.103</v>
       </c>
       <c r="I331" t="n">
-        <v>0.551</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="332">
@@ -17623,7 +17623,7 @@
         <v>0.299</v>
       </c>
       <c r="I333" t="n">
-        <v>0.965</v>
+        <v>1</v>
       </c>
     </row>
     <row r="334">
@@ -17771,7 +17771,7 @@
         <v>0.301</v>
       </c>
       <c r="I337" t="n">
-        <v>0.965</v>
+        <v>0.547</v>
       </c>
     </row>
     <row r="338">
@@ -17808,7 +17808,7 @@
         <v>0.216</v>
       </c>
       <c r="I338" t="n">
-        <v>0.979</v>
+        <v>0.831</v>
       </c>
     </row>
     <row r="339">
@@ -17845,7 +17845,7 @@
         <v>0.245</v>
       </c>
       <c r="I339" t="n">
-        <v>0.979</v>
+        <v>0.612</v>
       </c>
     </row>
     <row r="340">
@@ -17919,7 +17919,7 @@
         <v>1.34e-05</v>
       </c>
       <c r="I341" t="n">
-        <v>0.000214</v>
+        <v>5.03e-05</v>
       </c>
     </row>
     <row r="342">
@@ -18141,7 +18141,7 @@
         <v>0.383</v>
       </c>
       <c r="I347" t="n">
-        <v>1</v>
+        <v>0.754</v>
       </c>
     </row>
     <row r="348">
@@ -18178,7 +18178,7 @@
         <v>0.205</v>
       </c>
       <c r="I348" t="n">
-        <v>0.979</v>
+        <v>0.802</v>
       </c>
     </row>
     <row r="349">
@@ -18363,7 +18363,7 @@
         <v>0.35</v>
       </c>
       <c r="I353" t="n">
-        <v>1</v>
+        <v>0.656</v>
       </c>
     </row>
     <row r="354">
@@ -18400,7 +18400,7 @@
         <v>0.234</v>
       </c>
       <c r="I354" t="n">
-        <v>0.828</v>
+        <v>0.8149999999999999</v>
       </c>
     </row>
     <row r="355">
@@ -18511,7 +18511,7 @@
         <v>0.00466</v>
       </c>
       <c r="I357" t="n">
-        <v>0.0746</v>
+        <v>0.0175</v>
       </c>
     </row>
     <row r="358">
@@ -18659,7 +18659,7 @@
         <v>0.242</v>
       </c>
       <c r="I361" t="n">
-        <v>0.828</v>
+        <v>0.907</v>
       </c>
     </row>
     <row r="362">
@@ -18733,7 +18733,7 @@
         <v>0.208</v>
       </c>
       <c r="I363" t="n">
-        <v>0.828</v>
+        <v>1</v>
       </c>
     </row>
     <row r="364">
@@ -18807,7 +18807,7 @@
         <v>0.405</v>
       </c>
       <c r="I365" t="n">
-        <v>1</v>
+        <v>0.868</v>
       </c>
     </row>
     <row r="366">
@@ -18881,7 +18881,7 @@
         <v>0.605</v>
       </c>
       <c r="I367" t="n">
-        <v>1</v>
+        <v>0.826</v>
       </c>
     </row>
     <row r="368">
@@ -18955,7 +18955,7 @@
         <v>0.259</v>
       </c>
       <c r="I369" t="n">
-        <v>0.828</v>
+        <v>0.486</v>
       </c>
     </row>
     <row r="370">
@@ -18992,7 +18992,7 @@
         <v>0.75</v>
       </c>
       <c r="I370" t="n">
-        <v>0.919</v>
+        <v>0.984</v>
       </c>
     </row>
     <row r="371">
@@ -19029,7 +19029,7 @@
         <v>0.158</v>
       </c>
       <c r="I371" t="n">
-        <v>0.489</v>
+        <v>0.339</v>
       </c>
     </row>
     <row r="372">
@@ -19103,7 +19103,7 @@
         <v>1.04e-08</v>
       </c>
       <c r="I373" t="n">
-        <v>1.66e-07</v>
+        <v>3.9e-08</v>
       </c>
     </row>
     <row r="374">
@@ -19140,7 +19140,7 @@
         <v>0.427</v>
       </c>
       <c r="I374" t="n">
-        <v>0.847</v>
+        <v>1</v>
       </c>
     </row>
     <row r="375">
@@ -19177,7 +19177,7 @@
         <v>0.713</v>
       </c>
       <c r="I375" t="n">
-        <v>0.919</v>
+        <v>1</v>
       </c>
     </row>
     <row r="376">
@@ -19214,7 +19214,7 @@
         <v>0.348</v>
       </c>
       <c r="I376" t="n">
-        <v>0.796</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="377">
@@ -19251,7 +19251,7 @@
         <v>0.0584</v>
       </c>
       <c r="I377" t="n">
-        <v>0.336</v>
+        <v>0.219</v>
       </c>
     </row>
     <row r="378">
@@ -19288,7 +19288,7 @@
         <v>0.804</v>
       </c>
       <c r="I378" t="n">
-        <v>0.919</v>
+        <v>0.928</v>
       </c>
     </row>
     <row r="379">
@@ -19325,7 +19325,7 @@
         <v>0.0761</v>
       </c>
       <c r="I379" t="n">
-        <v>0.336</v>
+        <v>0.5620000000000001</v>
       </c>
     </row>
     <row r="380">
@@ -19362,7 +19362,7 @@
         <v>0.804</v>
       </c>
       <c r="I380" t="n">
-        <v>0.919</v>
+        <v>1</v>
       </c>
     </row>
     <row r="381">
@@ -19399,7 +19399,7 @@
         <v>0.183</v>
       </c>
       <c r="I381" t="n">
-        <v>0.489</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="382">
@@ -19473,7 +19473,7 @@
         <v>0.476</v>
       </c>
       <c r="I383" t="n">
-        <v>0.847</v>
+        <v>1</v>
       </c>
     </row>
     <row r="384">
@@ -19510,7 +19510,7 @@
         <v>0.787</v>
       </c>
       <c r="I384" t="n">
-        <v>0.919</v>
+        <v>1</v>
       </c>
     </row>
     <row r="385">
@@ -19547,7 +19547,7 @@
         <v>0.08400000000000001</v>
       </c>
       <c r="I385" t="n">
-        <v>0.336</v>
+        <v>0.158</v>
       </c>
     </row>
     <row r="386">
@@ -19621,7 +19621,7 @@
         <v>0.299</v>
       </c>
       <c r="I387" t="n">
-        <v>1</v>
+        <v>0.448</v>
       </c>
     </row>
     <row r="388">
@@ -20139,7 +20139,7 @@
         <v>0.0182</v>
       </c>
       <c r="I401" t="n">
-        <v>0.292</v>
+        <v>0.273</v>
       </c>
     </row>
     <row r="402">
@@ -20176,7 +20176,7 @@
         <v>0.224</v>
       </c>
       <c r="I402" t="n">
-        <v>1</v>
+        <v>0.831</v>
       </c>
     </row>
     <row r="403">
@@ -20213,7 +20213,7 @@
         <v>0.607</v>
       </c>
       <c r="I403" t="n">
-        <v>1</v>
+        <v>0.828</v>
       </c>
     </row>
     <row r="404">
@@ -20509,7 +20509,7 @@
         <v>0.6909999999999999</v>
       </c>
       <c r="I411" t="n">
-        <v>1</v>
+        <v>0.9419999999999999</v>
       </c>
     </row>
     <row r="412">
@@ -20546,7 +20546,7 @@
         <v>0.37</v>
       </c>
       <c r="I412" t="n">
-        <v>1</v>
+        <v>0.802</v>
       </c>
     </row>
     <row r="413">
@@ -20731,7 +20731,7 @@
         <v>0.122</v>
       </c>
       <c r="I417" t="n">
-        <v>1</v>
+        <v>0.608</v>
       </c>
     </row>
     <row r="418">
@@ -20768,7 +20768,7 @@
         <v>0.0219</v>
       </c>
       <c r="I418" t="n">
-        <v>0.175</v>
+        <v>0.329</v>
       </c>
     </row>
     <row r="419">
@@ -21027,7 +21027,7 @@
         <v>0.5669999999999999</v>
       </c>
       <c r="I425" t="n">
-        <v>1</v>
+        <v>0.945</v>
       </c>
     </row>
     <row r="426">
@@ -21175,7 +21175,7 @@
         <v>0.405</v>
       </c>
       <c r="I429" t="n">
-        <v>1</v>
+        <v>0.868</v>
       </c>
     </row>
     <row r="430">
@@ -21249,7 +21249,7 @@
         <v>0.342</v>
       </c>
       <c r="I431" t="n">
-        <v>1</v>
+        <v>0.826</v>
       </c>
     </row>
     <row r="432">
@@ -21323,7 +21323,7 @@
         <v>0.0134</v>
       </c>
       <c r="I433" t="n">
-        <v>0.175</v>
+        <v>0.101</v>
       </c>
     </row>
     <row r="434">
@@ -21360,7 +21360,7 @@
         <v>0.553</v>
       </c>
       <c r="I434" t="n">
-        <v>0.904</v>
+        <v>0.984</v>
       </c>
     </row>
     <row r="435">
@@ -21397,7 +21397,7 @@
         <v>0.415</v>
       </c>
       <c r="I435" t="n">
-        <v>0.904</v>
+        <v>0.6919999999999999</v>
       </c>
     </row>
     <row r="436">
@@ -21471,7 +21471,7 @@
         <v>0.481</v>
       </c>
       <c r="I437" t="n">
-        <v>0.904</v>
+        <v>0.722</v>
       </c>
     </row>
     <row r="438">
@@ -21508,7 +21508,7 @@
         <v>0.604</v>
       </c>
       <c r="I438" t="n">
-        <v>0.904</v>
+        <v>1</v>
       </c>
     </row>
     <row r="439">
@@ -21545,7 +21545,7 @@
         <v>0.313</v>
       </c>
       <c r="I439" t="n">
-        <v>0.904</v>
+        <v>1</v>
       </c>
     </row>
     <row r="440">
@@ -21582,7 +21582,7 @@
         <v>0.737</v>
       </c>
       <c r="I440" t="n">
-        <v>0.907</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="441">
@@ -21619,7 +21619,7 @@
         <v>0.321</v>
       </c>
       <c r="I441" t="n">
-        <v>0.904</v>
+        <v>0.535</v>
       </c>
     </row>
     <row r="442">
@@ -21656,7 +21656,7 @@
         <v>0.622</v>
       </c>
       <c r="I442" t="n">
-        <v>0.904</v>
+        <v>0.928</v>
       </c>
     </row>
     <row r="443">
@@ -21693,7 +21693,7 @@
         <v>0.477</v>
       </c>
       <c r="I443" t="n">
-        <v>0.904</v>
+        <v>0.868</v>
       </c>
     </row>
     <row r="444">
@@ -21767,7 +21767,7 @@
         <v>0.462</v>
       </c>
       <c r="I445" t="n">
-        <v>0.904</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="446">
@@ -21841,7 +21841,7 @@
         <v>0.699</v>
       </c>
       <c r="I447" t="n">
-        <v>0.907</v>
+        <v>1</v>
       </c>
     </row>
     <row r="448">
@@ -21878,7 +21878,7 @@
         <v>0.396</v>
       </c>
       <c r="I448" t="n">
-        <v>0.904</v>
+        <v>1</v>
       </c>
     </row>
     <row r="449">
@@ -21915,7 +21915,7 @@
         <v>0.000829</v>
       </c>
       <c r="I449" t="n">
-        <v>0.0133</v>
+        <v>0.0124</v>
       </c>
     </row>
     <row r="450">
@@ -21989,7 +21989,7 @@
         <v>0.0523</v>
       </c>
       <c r="I451" t="n">
-        <v>0.419</v>
+        <v>0.131</v>
       </c>
     </row>
     <row r="452">
@@ -22063,7 +22063,7 @@
         <v>1.52e-14</v>
       </c>
       <c r="I453" t="n">
-        <v>2.44e-13</v>
+        <v>2.28e-13</v>
       </c>
     </row>
     <row r="454">
@@ -22100,7 +22100,7 @@
         <v>0.399</v>
       </c>
       <c r="I454" t="n">
-        <v>0.9409999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="455">
@@ -22248,7 +22248,7 @@
         <v>0.552</v>
       </c>
       <c r="I458" t="n">
-        <v>0.981</v>
+        <v>1</v>
       </c>
     </row>
     <row r="459">
@@ -22285,7 +22285,7 @@
         <v>0.288</v>
       </c>
       <c r="I459" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="460">
@@ -22322,7 +22322,7 @@
         <v>0.412</v>
       </c>
       <c r="I460" t="n">
-        <v>0.9409999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="461">
@@ -22359,7 +22359,7 @@
         <v>0.472</v>
       </c>
       <c r="I461" t="n">
-        <v>0.9429999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="462">
@@ -22433,7 +22433,7 @@
         <v>0.181</v>
       </c>
       <c r="I463" t="n">
-        <v>0.9409999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="464">
@@ -22507,7 +22507,7 @@
         <v>0.301</v>
       </c>
       <c r="I465" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.547</v>
       </c>
     </row>
     <row r="466">
@@ -22581,7 +22581,7 @@
         <v>0.245</v>
       </c>
       <c r="I467" t="n">
-        <v>1</v>
+        <v>0.612</v>
       </c>
     </row>
     <row r="468">
@@ -22655,7 +22655,7 @@
         <v>2.65e-06</v>
       </c>
       <c r="I469" t="n">
-        <v>4.25e-05</v>
+        <v>2.82e-05</v>
       </c>
     </row>
     <row r="470">
@@ -22877,7 +22877,7 @@
         <v>0.402</v>
       </c>
       <c r="I475" t="n">
-        <v>1</v>
+        <v>0.754</v>
       </c>
     </row>
     <row r="476">
@@ -23099,7 +23099,7 @@
         <v>0.35</v>
       </c>
       <c r="I481" t="n">
-        <v>1</v>
+        <v>0.656</v>
       </c>
     </row>
     <row r="482">
@@ -23247,7 +23247,7 @@
         <v>0.00466</v>
       </c>
       <c r="I485" t="n">
-        <v>0.0746</v>
+        <v>0.0175</v>
       </c>
     </row>
     <row r="486">
@@ -23395,7 +23395,7 @@
         <v>0.5669999999999999</v>
       </c>
       <c r="I489" t="n">
-        <v>1</v>
+        <v>0.945</v>
       </c>
     </row>
     <row r="490">
@@ -23617,7 +23617,7 @@
         <v>0.182</v>
       </c>
       <c r="I495" t="n">
-        <v>1</v>
+        <v>0.826</v>
       </c>
     </row>
     <row r="496">
@@ -23691,7 +23691,7 @@
         <v>0.259</v>
       </c>
       <c r="I497" t="n">
-        <v>1</v>
+        <v>0.486</v>
       </c>
     </row>
     <row r="498">
@@ -23728,7 +23728,7 @@
         <v>0.776</v>
       </c>
       <c r="I498" t="n">
-        <v>0.975</v>
+        <v>0.984</v>
       </c>
     </row>
     <row r="499">
@@ -23765,7 +23765,7 @@
         <v>0.158</v>
       </c>
       <c r="I499" t="n">
-        <v>0.631</v>
+        <v>0.339</v>
       </c>
     </row>
     <row r="500">
@@ -23839,7 +23839,7 @@
         <v>1.18e-09</v>
       </c>
       <c r="I501" t="n">
-        <v>1.88e-08</v>
+        <v>1.66e-08</v>
       </c>
     </row>
     <row r="502">
@@ -23876,7 +23876,7 @@
         <v>0.427</v>
       </c>
       <c r="I502" t="n">
-        <v>0.768</v>
+        <v>1</v>
       </c>
     </row>
     <row r="503">
@@ -23913,7 +23913,7 @@
         <v>0.713</v>
       </c>
       <c r="I503" t="n">
-        <v>0.975</v>
+        <v>1</v>
       </c>
     </row>
     <row r="504">
@@ -23987,7 +23987,7 @@
         <v>0.321</v>
       </c>
       <c r="I505" t="n">
-        <v>0.768</v>
+        <v>0.535</v>
       </c>
     </row>
     <row r="506">
@@ -24024,7 +24024,7 @@
         <v>0.409</v>
       </c>
       <c r="I506" t="n">
-        <v>0.768</v>
+        <v>0.928</v>
       </c>
     </row>
     <row r="507">
@@ -24061,7 +24061,7 @@
         <v>0.225</v>
       </c>
       <c r="I507" t="n">
-        <v>0.719</v>
+        <v>0.5620000000000001</v>
       </c>
     </row>
     <row r="508">
@@ -24098,7 +24098,7 @@
         <v>0.452</v>
       </c>
       <c r="I508" t="n">
-        <v>0.768</v>
+        <v>1</v>
       </c>
     </row>
     <row r="509">
@@ -24135,7 +24135,7 @@
         <v>0.48</v>
       </c>
       <c r="I509" t="n">
-        <v>0.768</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="510">
@@ -24209,7 +24209,7 @@
         <v>0.107</v>
       </c>
       <c r="I511" t="n">
-        <v>0.571</v>
+        <v>0.802</v>
       </c>
     </row>
     <row r="512">
@@ -24246,7 +24246,7 @@
         <v>0.792</v>
       </c>
       <c r="I512" t="n">
-        <v>0.975</v>
+        <v>1</v>
       </c>
     </row>
     <row r="513">
@@ -24283,7 +24283,7 @@
         <v>0.08400000000000001</v>
       </c>
       <c r="I513" t="n">
-        <v>0.571</v>
+        <v>0.158</v>
       </c>
     </row>
     <row r="514">
@@ -24357,7 +24357,7 @@
         <v>0.0523</v>
       </c>
       <c r="I515" t="n">
-        <v>0.837</v>
+        <v>0.131</v>
       </c>
     </row>
     <row r="516">
@@ -24875,7 +24875,7 @@
         <v>0.301</v>
       </c>
       <c r="I529" t="n">
-        <v>1</v>
+        <v>0.547</v>
       </c>
     </row>
     <row r="530">
@@ -24912,7 +24912,7 @@
         <v>0.277</v>
       </c>
       <c r="I530" t="n">
-        <v>1</v>
+        <v>0.831</v>
       </c>
     </row>
     <row r="531">
@@ -24949,7 +24949,7 @@
         <v>0.245</v>
       </c>
       <c r="I531" t="n">
-        <v>1</v>
+        <v>0.612</v>
       </c>
     </row>
     <row r="532">
@@ -25282,7 +25282,7 @@
         <v>0.42</v>
       </c>
       <c r="I540" t="n">
-        <v>1</v>
+        <v>0.802</v>
       </c>
     </row>
     <row r="541">
@@ -25467,7 +25467,7 @@
         <v>0.35</v>
       </c>
       <c r="I545" t="n">
-        <v>1</v>
+        <v>0.656</v>
       </c>
     </row>
     <row r="546">
@@ -25504,7 +25504,7 @@
         <v>0.489</v>
       </c>
       <c r="I546" t="n">
-        <v>1</v>
+        <v>0.8149999999999999</v>
       </c>
     </row>
     <row r="547">
@@ -26059,7 +26059,7 @@
         <v>0.259</v>
       </c>
       <c r="I561" t="n">
-        <v>1</v>
+        <v>0.486</v>
       </c>
     </row>
     <row r="562">
@@ -26096,7 +26096,7 @@
         <v>0.746</v>
       </c>
       <c r="I562" t="n">
-        <v>1</v>
+        <v>0.984</v>
       </c>
     </row>
     <row r="563">
@@ -26133,7 +26133,7 @@
         <v>0.158</v>
       </c>
       <c r="I563" t="n">
-        <v>1</v>
+        <v>0.339</v>
       </c>
     </row>
     <row r="564">
@@ -26355,7 +26355,7 @@
         <v>0.628</v>
       </c>
       <c r="I569" t="n">
-        <v>1</v>
+        <v>0.9419999999999999</v>
       </c>
     </row>
     <row r="570">
@@ -26392,7 +26392,7 @@
         <v>0.796</v>
       </c>
       <c r="I570" t="n">
-        <v>1</v>
+        <v>0.928</v>
       </c>
     </row>
     <row r="571">
@@ -26503,7 +26503,7 @@
         <v>0.711</v>
       </c>
       <c r="I573" t="n">
-        <v>1</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="574">
@@ -26651,7 +26651,7 @@
         <v>0.08400000000000001</v>
       </c>
       <c r="I577" t="n">
-        <v>1</v>
+        <v>0.158</v>
       </c>
     </row>
     <row r="578">
@@ -26725,7 +26725,7 @@
         <v>0.145</v>
       </c>
       <c r="I579" t="n">
-        <v>0.719</v>
+        <v>0.272</v>
       </c>
     </row>
     <row r="580">
@@ -27021,7 +27021,7 @@
         <v>0.18</v>
       </c>
       <c r="I587" t="n">
-        <v>0.719</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="588">
@@ -27058,7 +27058,7 @@
         <v>0.08400000000000001</v>
       </c>
       <c r="I588" t="n">
-        <v>0.719</v>
+        <v>1</v>
       </c>
     </row>
     <row r="589">
@@ -27243,7 +27243,7 @@
         <v>0.12</v>
       </c>
       <c r="I593" t="n">
-        <v>0.719</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="594">
@@ -27280,7 +27280,7 @@
         <v>0.481</v>
       </c>
       <c r="I594" t="n">
-        <v>1</v>
+        <v>0.913</v>
       </c>
     </row>
     <row r="595">
@@ -27317,7 +27317,7 @@
         <v>0.329</v>
       </c>
       <c r="I595" t="n">
-        <v>1</v>
+        <v>0.705</v>
       </c>
     </row>
     <row r="596">
@@ -27613,7 +27613,7 @@
         <v>0.391</v>
       </c>
       <c r="I603" t="n">
-        <v>1</v>
+        <v>0.754</v>
       </c>
     </row>
     <row r="604">
@@ -27650,7 +27650,7 @@
         <v>0.187</v>
       </c>
       <c r="I604" t="n">
-        <v>1</v>
+        <v>0.802</v>
       </c>
     </row>
     <row r="605">
@@ -27835,7 +27835,7 @@
         <v>0.119</v>
       </c>
       <c r="I609" t="n">
-        <v>1</v>
+        <v>0.608</v>
       </c>
     </row>
     <row r="610">
@@ -28131,7 +28131,7 @@
         <v>0.5669999999999999</v>
       </c>
       <c r="I617" t="n">
-        <v>1</v>
+        <v>0.945</v>
       </c>
     </row>
     <row r="618">
@@ -28279,7 +28279,7 @@
         <v>0.405</v>
       </c>
       <c r="I621" t="n">
-        <v>1</v>
+        <v>0.868</v>
       </c>
     </row>
     <row r="622">
@@ -28353,7 +28353,7 @@
         <v>0.605</v>
       </c>
       <c r="I623" t="n">
-        <v>1</v>
+        <v>0.826</v>
       </c>
     </row>
     <row r="624">
@@ -28427,7 +28427,7 @@
         <v>0.259</v>
       </c>
       <c r="I625" t="n">
-        <v>1</v>
+        <v>0.486</v>
       </c>
     </row>
     <row r="626">
@@ -28464,7 +28464,7 @@
         <v>0.743</v>
       </c>
       <c r="I626" t="n">
-        <v>1</v>
+        <v>0.984</v>
       </c>
     </row>
     <row r="627">
@@ -28501,7 +28501,7 @@
         <v>0.367</v>
       </c>
       <c r="I627" t="n">
-        <v>1</v>
+        <v>0.6879999999999999</v>
       </c>
     </row>
     <row r="628">
@@ -28575,7 +28575,7 @@
         <v>0.481</v>
       </c>
       <c r="I629" t="n">
-        <v>1</v>
+        <v>0.722</v>
       </c>
     </row>
     <row r="630">
@@ -28686,7 +28686,7 @@
         <v>0.731</v>
       </c>
       <c r="I632" t="n">
-        <v>1</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="633">
@@ -28723,7 +28723,7 @@
         <v>0.321</v>
       </c>
       <c r="I633" t="n">
-        <v>1</v>
+        <v>0.535</v>
       </c>
     </row>
     <row r="634">
@@ -28760,7 +28760,7 @@
         <v>0.594</v>
       </c>
       <c r="I634" t="n">
-        <v>1</v>
+        <v>0.928</v>
       </c>
     </row>
     <row r="635">
@@ -28797,7 +28797,7 @@
         <v>0.136</v>
       </c>
       <c r="I635" t="n">
-        <v>0.727</v>
+        <v>0.5620000000000001</v>
       </c>
     </row>
     <row r="636">
@@ -28834,7 +28834,7 @@
         <v>0.107</v>
       </c>
       <c r="I636" t="n">
-        <v>0.727</v>
+        <v>1</v>
       </c>
     </row>
     <row r="637">
@@ -28871,7 +28871,7 @@
         <v>0.462</v>
       </c>
       <c r="I637" t="n">
-        <v>1</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="638">
@@ -29019,7 +29019,7 @@
         <v>0.0421</v>
       </c>
       <c r="I641" t="n">
-        <v>0.673</v>
+        <v>0.126</v>
       </c>
     </row>
     <row r="642">
@@ -29611,7 +29611,7 @@
         <v>0.604</v>
       </c>
       <c r="I657" t="n">
-        <v>1</v>
+        <v>0.647</v>
       </c>
     </row>
     <row r="658">
@@ -30203,7 +30203,7 @@
         <v>0.768</v>
       </c>
       <c r="I673" t="n">
-        <v>1</v>
+        <v>0.823</v>
       </c>
     </row>
     <row r="674">
@@ -30832,7 +30832,7 @@
         <v>0.776</v>
       </c>
       <c r="I690" t="n">
-        <v>1</v>
+        <v>0.984</v>
       </c>
     </row>
     <row r="691">
@@ -31054,7 +31054,7 @@
         <v>0.705</v>
       </c>
       <c r="I696" t="n">
-        <v>1</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="697">
@@ -31128,7 +31128,7 @@
         <v>0.3</v>
       </c>
       <c r="I698" t="n">
-        <v>1</v>
+        <v>0.928</v>
       </c>
     </row>
     <row r="699">
@@ -31165,7 +31165,7 @@
         <v>0.536</v>
       </c>
       <c r="I699" t="n">
-        <v>1</v>
+        <v>0.868</v>
       </c>
     </row>
     <row r="700">
@@ -31239,7 +31239,7 @@
         <v>0.752</v>
       </c>
       <c r="I701" t="n">
-        <v>1</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="702">
@@ -31387,7 +31387,7 @@
         <v>0.65</v>
       </c>
       <c r="I705" t="n">
-        <v>1</v>
+        <v>0.696</v>
       </c>
     </row>
     <row r="706">
@@ -31979,7 +31979,7 @@
         <v>0.435</v>
       </c>
       <c r="I721" t="n">
-        <v>1</v>
+        <v>0.547</v>
       </c>
     </row>
     <row r="722">
@@ -32349,7 +32349,7 @@
         <v>0.238</v>
       </c>
       <c r="I731" t="n">
-        <v>1</v>
+        <v>0.754</v>
       </c>
     </row>
     <row r="732">
@@ -32571,7 +32571,7 @@
         <v>0.763</v>
       </c>
       <c r="I737" t="n">
-        <v>1</v>
+        <v>0.823</v>
       </c>
     </row>
     <row r="738">
@@ -33089,7 +33089,7 @@
         <v>0.661</v>
       </c>
       <c r="I751" t="n">
-        <v>1</v>
+        <v>0.826</v>
       </c>
     </row>
     <row r="752">
@@ -33422,7 +33422,7 @@
         <v>0.712</v>
       </c>
       <c r="I760" t="n">
-        <v>1</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="761">
@@ -33496,7 +33496,7 @@
         <v>0.787</v>
       </c>
       <c r="I762" t="n">
-        <v>1</v>
+        <v>0.928</v>
       </c>
     </row>
     <row r="763">
@@ -33607,7 +33607,7 @@
         <v>0.734</v>
       </c>
       <c r="I765" t="n">
-        <v>1</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="766">
@@ -33755,7 +33755,7 @@
         <v>0.494</v>
       </c>
       <c r="I769" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
     </row>
     <row r="770">
@@ -34347,7 +34347,7 @@
         <v>0.796</v>
       </c>
       <c r="I785" t="n">
-        <v>1</v>
+        <v>0.796</v>
       </c>
     </row>
     <row r="786">
@@ -34717,7 +34717,7 @@
         <v>0.243</v>
       </c>
       <c r="I795" t="n">
-        <v>1</v>
+        <v>0.754</v>
       </c>
     </row>
     <row r="796">
@@ -34976,7 +34976,7 @@
         <v>0.609</v>
       </c>
       <c r="I802" t="n">
-        <v>1</v>
+        <v>0.913</v>
       </c>
     </row>
     <row r="803">
@@ -35457,7 +35457,7 @@
         <v>0.661</v>
       </c>
       <c r="I815" t="n">
-        <v>1</v>
+        <v>0.826</v>
       </c>
     </row>
     <row r="816">
@@ -35568,7 +35568,7 @@
         <v>0.594</v>
       </c>
       <c r="I818" t="n">
-        <v>1</v>
+        <v>0.984</v>
       </c>
     </row>
     <row r="819">
@@ -35605,7 +35605,7 @@
         <v>0.5590000000000001</v>
       </c>
       <c r="I819" t="n">
-        <v>1</v>
+        <v>0.839</v>
       </c>
     </row>
     <row r="820">
@@ -35679,7 +35679,7 @@
         <v>0.481</v>
       </c>
       <c r="I821" t="n">
-        <v>1</v>
+        <v>0.722</v>
       </c>
     </row>
     <row r="822">
@@ -35790,7 +35790,7 @@
         <v>0.712</v>
       </c>
       <c r="I824" t="n">
-        <v>1</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="825">
@@ -35975,7 +35975,7 @@
         <v>0.765</v>
       </c>
       <c r="I829" t="n">
-        <v>1</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="830">
@@ -36123,7 +36123,7 @@
         <v>0.8179999999999999</v>
       </c>
       <c r="I833" t="n">
-        <v>1</v>
+        <v>0.8179999999999999</v>
       </c>
     </row>
     <row r="834">
@@ -36715,7 +36715,7 @@
         <v>0.435</v>
       </c>
       <c r="I849" t="n">
-        <v>1</v>
+        <v>0.547</v>
       </c>
     </row>
     <row r="850">
@@ -37307,7 +37307,7 @@
         <v>0.768</v>
       </c>
       <c r="I865" t="n">
-        <v>1</v>
+        <v>0.823</v>
       </c>
     </row>
     <row r="866">
@@ -37936,7 +37936,7 @@
         <v>0.787</v>
       </c>
       <c r="I882" t="n">
-        <v>1</v>
+        <v>0.984</v>
       </c>
     </row>
     <row r="883">
@@ -38158,7 +38158,7 @@
         <v>0.476</v>
       </c>
       <c r="I888" t="n">
-        <v>1</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="889">
@@ -38232,7 +38232,7 @@
         <v>0.787</v>
       </c>
       <c r="I890" t="n">
-        <v>1</v>
+        <v>0.928</v>
       </c>
     </row>
     <row r="891">
@@ -38491,7 +38491,7 @@
         <v>0.506</v>
       </c>
       <c r="I897" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
     </row>
     <row r="898">
@@ -38565,7 +38565,7 @@
         <v>0.353</v>
       </c>
       <c r="I899" t="n">
-        <v>1</v>
+        <v>0.481</v>
       </c>
     </row>
     <row r="900">
@@ -39083,7 +39083,7 @@
         <v>0.435</v>
       </c>
       <c r="I913" t="n">
-        <v>1</v>
+        <v>0.547</v>
       </c>
     </row>
     <row r="914">
@@ -39120,7 +39120,7 @@
         <v>0.44</v>
       </c>
       <c r="I914" t="n">
-        <v>1</v>
+        <v>0.913</v>
       </c>
     </row>
     <row r="915">
@@ -39157,7 +39157,7 @@
         <v>0.486</v>
       </c>
       <c r="I915" t="n">
-        <v>1</v>
+        <v>0.828</v>
       </c>
     </row>
     <row r="916">
@@ -39675,7 +39675,7 @@
         <v>0.526</v>
       </c>
       <c r="I929" t="n">
-        <v>1</v>
+        <v>0.823</v>
       </c>
     </row>
     <row r="930">
@@ -39712,7 +39712,7 @@
         <v>0.348</v>
       </c>
       <c r="I930" t="n">
-        <v>1</v>
+        <v>0.8149999999999999</v>
       </c>
     </row>
     <row r="931">
@@ -39786,7 +39786,7 @@
         <v>0.021</v>
       </c>
       <c r="I932" t="n">
-        <v>0.336</v>
+        <v>0.315</v>
       </c>
     </row>
     <row r="933">
@@ -40008,7 +40008,7 @@
         <v>0.103</v>
       </c>
       <c r="I938" t="n">
-        <v>0.827</v>
+        <v>1</v>
       </c>
     </row>
     <row r="939">
@@ -40193,7 +40193,7 @@
         <v>0.407</v>
       </c>
       <c r="I943" t="n">
-        <v>1</v>
+        <v>0.826</v>
       </c>
     </row>
     <row r="944">
@@ -40341,7 +40341,7 @@
         <v>0.103</v>
       </c>
       <c r="I947" t="n">
-        <v>0.547</v>
+        <v>0.339</v>
       </c>
     </row>
     <row r="948">
@@ -40378,7 +40378,7 @@
         <v>0.0147</v>
       </c>
       <c r="I948" t="n">
-        <v>0.235</v>
+        <v>0.221</v>
       </c>
     </row>
     <row r="949">
@@ -40415,7 +40415,7 @@
         <v>0.203</v>
       </c>
       <c r="I949" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.609</v>
       </c>
     </row>
     <row r="950">
@@ -40526,7 +40526,7 @@
         <v>0.3</v>
       </c>
       <c r="I952" t="n">
-        <v>0.96</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="953">
@@ -40600,7 +40600,7 @@
         <v>0.0489</v>
       </c>
       <c r="I954" t="n">
-        <v>0.391</v>
+        <v>0.734</v>
       </c>
     </row>
     <row r="955">
@@ -40637,7 +40637,7 @@
         <v>0.579</v>
       </c>
       <c r="I955" t="n">
-        <v>1</v>
+        <v>0.868</v>
       </c>
     </row>
     <row r="956">
@@ -40711,7 +40711,7 @@
         <v>0.554</v>
       </c>
       <c r="I957" t="n">
-        <v>1</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="958">
@@ -40859,7 +40859,7 @@
         <v>0.628</v>
       </c>
       <c r="I961" t="n">
-        <v>1</v>
+        <v>0.696</v>
       </c>
     </row>
   </sheetData>

</xml_diff>